<commit_message>
Turn 2.5: Machine/Factory/Lab compounding architecture
Consolidate 10 tools → 5 (shorter descriptions, trust the model).
Kill calibration system (30-param schema was anti-bitter-lesson).
Add persistent event log (append-only JSONL) for Factory compounding.
Wire aggregate signal into read_constitution + mode activations so
every conversation feeds the general compounding loop automatically.
Add Lab loop: models observe system effectiveness from aggregate
signal and log observations for CTO cold start to act on.

Machine (specific): Constitution + feedback, per-Author, automatic.
Factory (general): event log → model adjusts, cross-Author, automatic.
Lab (system): models + CTO evaluate and improve Machine/Factory.

All three: meta (unstructured data appreciates with model quality),
bitter lesson aligned (general methods, no hand-crafted rules).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Numbers.xlsx
+++ b/docs/Numbers.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="149">
   <si>
     <t xml:space="preserve">Alexandria — Financial Model</t>
   </si>
@@ -257,22 +257,22 @@
     <t xml:space="preserve">MARKETING / ADS</t>
   </si>
   <si>
-    <t xml:space="preserve">Year 1 ad spend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zero — organic only via kin mechanic + founder network</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year 2+ ad spend (monthly, if funded)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modest — Claude community ads, targeted social. Only if funded.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year 2+ engineering hire (monthly, if funded)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Part-time engineer, deferred until funded</t>
+    <t xml:space="preserve">Year 1 ad spend (monthly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modest — brand seeding, community, events. ~$500/mo from raise.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 2+ ad spend (monthly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scales modestly with revenue. Ads, events, merch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineering hire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None. Solo founder + AI agents. No hires planned.</t>
   </si>
   <si>
     <t xml:space="preserve">EXIT / VALUATION</t>
@@ -413,9 +413,6 @@
     <t xml:space="preserve">Ads / marketing</t>
   </si>
   <si>
-    <t xml:space="preserve">Engineering hire (if funded)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Founder living costs</t>
   </si>
   <si>
@@ -449,7 +446,7 @@
     <t xml:space="preserve">Implied exit valuation</t>
   </si>
   <si>
-    <t xml:space="preserve">Investor return on $500K at 20% equity</t>
+    <t xml:space="preserve">Investor return on $50K at 5% equity</t>
   </si>
   <si>
     <t xml:space="preserve">Return multiple (MOM)</t>
@@ -1449,7 +1446,7 @@
         <v>78</v>
       </c>
       <c r="B58" s="6" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="C58" s="7" t="s">
         <v>79</v>
@@ -1471,7 +1468,7 @@
         <v>82</v>
       </c>
       <c r="B60" s="6" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="C60" s="7" t="s">
         <v>83</v>
@@ -2074,7 +2071,7 @@
         <v>129</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="C29" s="15" t="n">
         <f aca="false">1000*12</f>
@@ -2095,31 +2092,27 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>130</v>
+        <v>82</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C30" s="15" t="n">
-        <f aca="false">8000*12</f>
-        <v>96000</v>
+        <v>0</v>
       </c>
       <c r="D30" s="15" t="n">
-        <f aca="false">8000*12</f>
-        <v>96000</v>
+        <v>0</v>
       </c>
       <c r="E30" s="15" t="n">
-        <f aca="false">8000*12</f>
-        <v>96000</v>
+        <v>0</v>
       </c>
       <c r="F30" s="15" t="n">
-        <f aca="false">8000*12</f>
-        <v>96000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B31" s="15" t="n">
         <v>3360</v>
@@ -2139,112 +2132,112 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B32" s="16" t="n">
         <f aca="false">SUM(B23:B31)</f>
-        <v>23870.36</v>
+        <v>29870.36</v>
       </c>
       <c r="C32" s="16" t="n">
         <f aca="false">SUM(C23:C31)</f>
-        <v>150856.54</v>
+        <v>54856.54</v>
       </c>
       <c r="D32" s="16" t="n">
         <f aca="false">SUM(D23:D31)</f>
-        <v>197961.222</v>
+        <v>101961.222</v>
       </c>
       <c r="E32" s="16" t="n">
         <f aca="false">SUM(E23:E31)</f>
-        <v>290816.5486</v>
+        <v>194816.5486</v>
       </c>
       <c r="F32" s="16" t="n">
         <f aca="false">SUM(F23:F31)</f>
-        <v>400767.17878</v>
+        <v>304767.17878</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B35" s="16" t="n">
         <f aca="false">B20-B32</f>
-        <v>186969.64</v>
+        <v>180969.64</v>
       </c>
       <c r="C35" s="16" t="n">
         <f aca="false">C20-C32</f>
-        <v>384403.46</v>
+        <v>480403.46</v>
       </c>
       <c r="D35" s="16" t="n">
         <f aca="false">D20-D32</f>
-        <v>1112556.778</v>
+        <v>1208556.778</v>
       </c>
       <c r="E35" s="16" t="n">
         <f aca="false">E20-E32</f>
-        <v>2359096.8514</v>
+        <v>2455096.8514</v>
       </c>
       <c r="F35" s="16" t="n">
         <f aca="false">F20-F32</f>
-        <v>4178806.64122</v>
+        <v>4274806.64122</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B36" s="15" t="n">
         <f aca="false">B35</f>
-        <v>186969.64</v>
+        <v>180969.64</v>
       </c>
       <c r="C36" s="15" t="n">
         <f aca="false">B36+C35</f>
-        <v>571373.1</v>
+        <v>661373.1</v>
       </c>
       <c r="D36" s="15" t="n">
         <f aca="false">C36+D35</f>
-        <v>1683929.878</v>
+        <v>1869929.878</v>
       </c>
       <c r="E36" s="15" t="n">
         <f aca="false">D36+E35</f>
-        <v>4043026.7294</v>
+        <v>4325026.7294</v>
       </c>
       <c r="F36" s="15" t="n">
         <f aca="false">E36+F35</f>
-        <v>8221833.37062</v>
+        <v>8599833.37062</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B37" s="18" t="n">
         <f aca="false">IF(B20=0,0,B35/B20)</f>
-        <v>0.886784481123127</v>
+        <v>0.858326882944413</v>
       </c>
       <c r="C37" s="18" t="n">
         <f aca="false">IF(C20=0,0,C35/C20)</f>
-        <v>0.718162126816874</v>
+        <v>0.89751421738968</v>
       </c>
       <c r="D37" s="18" t="n">
         <f aca="false">IF(D20=0,0,D35/D20)</f>
-        <v>0.848944293783069</v>
+        <v>0.922197770652521</v>
       </c>
       <c r="E37" s="18" t="n">
         <f aca="false">IF(E20=0,0,E35/E20)</f>
-        <v>0.890254319782677</v>
+        <v>0.92648191876761</v>
       </c>
       <c r="F37" s="18" t="n">
         <f aca="false">IF(F20=0,0,F35/F20)</f>
-        <v>0.912488105982753</v>
+        <v>0.933450755297575</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B38" s="15" t="n">
         <f aca="false">B20</f>
@@ -2269,12 +2262,12 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B41" s="15" t="n">
         <f aca="false">F20</f>
@@ -2283,7 +2276,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B42" s="6" t="n">
         <v>20</v>
@@ -2291,7 +2284,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B43" s="16" t="n">
         <f aca="false">B41*B42</f>
@@ -2300,30 +2293,30 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B45" s="16" t="n">
-        <f aca="false">B43*0.2</f>
-        <v>18318295.28</v>
+        <f aca="false">B43*0.05</f>
+        <v>4579573.82</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B46" s="19" t="n">
-        <f aca="false">B45/500000</f>
-        <v>36.63659056</v>
+        <f aca="false">B45/50000</f>
+        <v>91.5914764</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>80</v>
@@ -2331,7 +2324,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>58</v>
@@ -2339,7 +2332,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>20</v>
@@ -2347,10 +2340,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
COO session sync: OAuth findings, tool activation research, doc updates
Major findings: OAuth invalid_grant is Claude platform bug (#21333).
Tool activation baseline is 20%, improves to 84% with proper
descriptions (4-6 sentences, explicit triggers, negative capability).
Blueprint updated: calibration → compounding architecture.
All investor docs updated for 5-tool architecture.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Numbers.xlsx
+++ b/docs/Numbers.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="155">
   <si>
     <t xml:space="preserve">Alexandria — Financial Model</t>
   </si>
@@ -80,13 +80,13 @@
     <t xml:space="preserve">Effective Sovereignty ARPU</t>
   </si>
   <si>
-    <t xml:space="preserve">Blended: 60% at $5, 40% at $10</t>
+    <t xml:space="preserve">Blended: 60% at $5, 40% at $10 = $7</t>
   </si>
   <si>
     <t xml:space="preserve">Effective Examined Life ARPU</t>
   </si>
   <si>
-    <t xml:space="preserve">Blended: 60% at $15, 40% at $20</t>
+    <t xml:space="preserve">Blended: 60% at $15, 40% at $20 = $17</t>
   </si>
   <si>
     <t xml:space="preserve">GROWTH</t>
@@ -149,10 +149,28 @@
     <t xml:space="preserve">$100/month</t>
   </si>
   <si>
+    <t xml:space="preserve">Railway Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCP server hosting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude API credits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API usage for MCP server and development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google AI Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video models + Google Drive storage</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total monthly operating costs</t>
   </si>
   <si>
-    <t xml:space="preserve">$120/month. Railway free. Domain owned. No other tools.</t>
+    <t xml:space="preserve">$210/month. Vercel + Claude Max + Claude API + Railway + Google AI Pro.</t>
   </si>
   <si>
     <t xml:space="preserve">Annual operating costs</t>
@@ -245,10 +263,16 @@
     <t xml:space="preserve">Living with a friend. No rent obligation.</t>
   </si>
   <si>
+    <t xml:space="preserve">Buffer / misc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal buffer</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total monthly founder costs</t>
   </si>
   <si>
-    <t xml:space="preserve">$280/month. Total burn with company: $400/month.</t>
+    <t xml:space="preserve">$290/month. Total burn with company: $500/month.</t>
   </si>
   <si>
     <t xml:space="preserve">Annual founder costs</t>
@@ -398,12 +422,6 @@
     <t xml:space="preserve">Claude Max 5x subscription</t>
   </si>
   <si>
-    <t xml:space="preserve">MCP server (Railway)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other tools &amp; services</t>
-  </si>
-  <si>
     <t xml:space="preserve">Stripe processing fees</t>
   </si>
   <si>
@@ -446,7 +464,7 @@
     <t xml:space="preserve">Implied exit valuation</t>
   </si>
   <si>
-    <t xml:space="preserve">Investor return on $50K at 5% equity</t>
+    <t xml:space="preserve">Investor return on $50K at ~1% equity ($5M pre-money)</t>
   </si>
   <si>
     <t xml:space="preserve">Return multiple (MOM)</t>
@@ -467,7 +485,7 @@
     <t xml:space="preserve">Total monthly burn</t>
   </si>
   <si>
-    <t xml:space="preserve">$400 ($120 company + $280 founder)</t>
+    <t xml:space="preserve">$500 ($210 company + $290 founder)</t>
   </si>
 </sst>
 </file>
@@ -673,7 +691,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -965,7 +983,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
@@ -1086,8 +1104,8 @@
         <v>18</v>
       </c>
       <c r="B15" s="8" t="n">
-        <f aca="false">B14*(1-B8)+B9*(1-B14)</f>
-        <v>1.6</v>
+        <f aca="false">B8*B14+B9*(1-B14)</f>
+        <v>7</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>19</v>
@@ -1098,8 +1116,8 @@
         <v>20</v>
       </c>
       <c r="B16" s="8" t="n">
-        <f aca="false">B10*(1-B14)+B11*(1-B14)</f>
-        <v>14</v>
+        <f aca="false">B10*B14+B11*(1-B14)</f>
+        <v>17</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>21</v>
@@ -1215,361 +1233,392 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="6"/>
-      <c r="C30" s="7"/>
+      <c r="A30" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="9"/>
-      <c r="C31" s="7"/>
+      <c r="A31" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="9"/>
-      <c r="C32" s="7"/>
+      <c r="A32" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B33" s="10" t="n">
-        <f aca="false">B28+B29</f>
-        <v>120</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>43</v>
-      </c>
+      <c r="B33" s="9"/>
+      <c r="C33" s="7"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B34" s="10" t="n">
-        <f aca="false">B33*12</f>
-        <v>1440</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
+        <v>210</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" s="10" t="n">
+        <f aca="false">B34*12</f>
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B37" s="6" t="n">
-        <v>500</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>47</v>
+      <c r="A37" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B40" s="6" t="n">
-        <v>800</v>
+        <v>150</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B41" s="6" t="n">
-        <v>150</v>
+        <v>800</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B42" s="6" t="n">
-        <v>1500</v>
+        <v>150</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B43" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B44" s="6" t="n">
         <v>500</v>
       </c>
-      <c r="C43" s="7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="B44" s="9" t="n">
+      <c r="C44" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B45" s="9" t="n">
         <v>1000</v>
       </c>
-      <c r="C44" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B45" s="10" t="n">
+      <c r="C45" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B46" s="10" t="n">
         <f aca="false">SUM(B37:B44)</f>
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B48" s="9" t="n">
-        <v>220</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>65</v>
+      <c r="A48" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B49" s="9" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B50" s="9" t="n">
         <v>0</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B51" s="9" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B52" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B53" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C52" s="7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="9"/>
-      <c r="C53" s="7"/>
+      <c r="C53" s="7" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B54" s="10" t="n">
-        <f aca="false">B48+B49+B50+B51+B52</f>
-        <v>280</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
+      </c>
+      <c r="B54" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B55" s="10" t="n">
-        <f aca="false">B54*12</f>
-        <v>3360</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
+        <v>290</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B56" s="10" t="n">
+        <f aca="false">B55*12</f>
+        <v>3480</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B58" s="6" t="n">
-        <v>500</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>79</v>
+      <c r="A58" s="4" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B59" s="6" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B60" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B61" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C60" s="7" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
+      <c r="C61" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B63" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C63" s="7" t="s">
-        <v>86</v>
+      <c r="A63" s="4" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B64" s="6" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B65" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="B65" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B66" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="C65" s="7" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
+      <c r="C66" s="7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B68" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C68" s="7" t="s">
-        <v>93</v>
+      <c r="A68" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B69" s="6" t="n">
-        <v>50000</v>
+        <v>2</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B70" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C70" s="7"/>
+        <v>50000</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B71" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="C71" s="7" t="s">
-        <v>98</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C71" s="7"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B72" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B73" s="6" t="n">
         <v>25000</v>
       </c>
-      <c r="C72" s="7" t="s">
-        <v>100</v>
+      <c r="C73" s="7" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1588,7 +1637,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
@@ -1597,34 +1646,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B5" s="13" t="n">
         <v>2000</v>
@@ -1644,7 +1693,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>0.08</v>
@@ -1664,7 +1713,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">B5*B6</f>
@@ -1689,7 +1738,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B8" s="6" t="n">
         <v>50</v>
@@ -1713,7 +1762,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B9" s="15" t="n">
         <f aca="false">B7+B8</f>
@@ -1738,7 +1787,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B10" s="16" t="n">
         <f aca="false">B5+B9</f>
@@ -1763,12 +1812,12 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B13" s="15" t="n">
         <f aca="false">B5*7*12</f>
@@ -1793,7 +1842,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B14" s="15" t="n">
         <f aca="false">B9*17*12</f>
@@ -1818,7 +1867,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B15" s="16" t="n">
         <f aca="false">B13+B14</f>
@@ -1843,7 +1892,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="B17" s="6" t="n">
         <v>0</v>
@@ -1863,7 +1912,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B18" s="6" t="n">
         <v>0</v>
@@ -1883,7 +1932,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B19" s="15" t="n">
         <f aca="false">B17+B18</f>
@@ -1908,7 +1957,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B20" s="16" t="n">
         <f aca="false">B15+B19</f>
@@ -1933,12 +1982,12 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B23" s="15" t="n">
         <f aca="false">20*12</f>
@@ -1963,7 +2012,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B24" s="15" t="n">
         <v>1200</v>
@@ -1983,367 +2032,391 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>125</v>
+        <v>42</v>
       </c>
       <c r="B25" s="15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="C25" s="15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="D25" s="15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="15" t="n">
-        <v>0</v>
+        <v>44</v>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>600</v>
+      </c>
+      <c r="C26" s="1" t="n">
+        <v>600</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>600</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>600</v>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>600</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>127</v>
+        <v>46</v>
       </c>
       <c r="B27" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="15" t="n">
         <f aca="false">B20*0.029+B10*0.3*12</f>
         <v>14070.36</v>
       </c>
-      <c r="C27" s="15" t="n">
+      <c r="C28" s="15" t="n">
         <f aca="false">C20*0.029+C10*0.3*12</f>
         <v>35556.54</v>
       </c>
-      <c r="D27" s="15" t="n">
+      <c r="D28" s="15" t="n">
         <f aca="false">D20*0.029+D10*0.3*12</f>
         <v>82661.222</v>
       </c>
-      <c r="E27" s="15" t="n">
+      <c r="E28" s="15" t="n">
         <f aca="false">E20*0.029+E10*0.3*12</f>
         <v>163016.5486</v>
       </c>
-      <c r="F27" s="15" t="n">
+      <c r="F28" s="15" t="n">
         <f aca="false">F20*0.029+F10*0.3*12</f>
         <v>272967.17878</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B28" s="13" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C28" s="13" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D28" s="13" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E28" s="13" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>3000</v>
-      </c>
-    </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B29" s="6" t="n">
+        <v>134</v>
+      </c>
+      <c r="B29" s="13" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C29" s="13" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B30" s="6" t="n">
         <v>6000</v>
       </c>
-      <c r="C29" s="15" t="n">
+      <c r="C30" s="15" t="n">
         <f aca="false">1000*12</f>
         <v>12000</v>
       </c>
-      <c r="D29" s="15" t="n">
+      <c r="D30" s="15" t="n">
         <f aca="false">1000*12</f>
         <v>12000</v>
       </c>
-      <c r="E29" s="15" t="n">
+      <c r="E30" s="15" t="n">
         <f aca="false">2000*12</f>
         <v>24000</v>
       </c>
-      <c r="F29" s="15" t="n">
+      <c r="F30" s="15" t="n">
         <f aca="false">2000*12</f>
         <v>24000</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B30" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B31" s="15" t="n">
-        <v>3360</v>
+        <v>90</v>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="C31" s="15" t="n">
-        <v>3360</v>
+        <v>0</v>
       </c>
       <c r="D31" s="15" t="n">
-        <v>3360</v>
+        <v>0</v>
       </c>
       <c r="E31" s="15" t="n">
-        <v>3360</v>
+        <v>0</v>
       </c>
       <c r="F31" s="15" t="n">
-        <v>3360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B32" s="16" t="n">
-        <f aca="false">SUM(B23:B31)</f>
-        <v>29870.36</v>
-      </c>
-      <c r="C32" s="16" t="n">
-        <f aca="false">SUM(C23:C31)</f>
-        <v>54856.54</v>
-      </c>
-      <c r="D32" s="16" t="n">
-        <f aca="false">SUM(D23:D31)</f>
-        <v>101961.222</v>
-      </c>
-      <c r="E32" s="16" t="n">
-        <f aca="false">SUM(E23:E31)</f>
-        <v>194816.5486</v>
-      </c>
-      <c r="F32" s="16" t="n">
-        <f aca="false">SUM(F23:F31)</f>
-        <v>304767.17878</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
+        <v>136</v>
+      </c>
+      <c r="B32" s="15" t="n">
+        <v>3480</v>
+      </c>
+      <c r="C32" s="15" t="n">
+        <v>3480</v>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>3480</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>3480</v>
+      </c>
+      <c r="F32" s="15" t="n">
+        <v>3480</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" s="16" t="n">
+        <f aca="false">SUM(B23:B32)</f>
+        <v>31070.36</v>
+      </c>
+      <c r="C33" s="16" t="n">
+        <f aca="false">SUM(C23:C32)</f>
+        <v>56056.54</v>
+      </c>
+      <c r="D33" s="16" t="n">
+        <f aca="false">SUM(D23:D32)</f>
+        <v>103161.222</v>
+      </c>
+      <c r="E33" s="16" t="n">
+        <f aca="false">SUM(E23:E32)</f>
+        <v>196016.5486</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <f aca="false">SUM(F23:F32)</f>
+        <v>305967.17878</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B35" s="16" t="n">
-        <f aca="false">B20-B32</f>
-        <v>180969.64</v>
-      </c>
-      <c r="C35" s="16" t="n">
-        <f aca="false">C20-C32</f>
-        <v>480403.46</v>
-      </c>
-      <c r="D35" s="16" t="n">
-        <f aca="false">D20-D32</f>
-        <v>1208556.778</v>
-      </c>
-      <c r="E35" s="16" t="n">
-        <f aca="false">E20-E32</f>
-        <v>2455096.8514</v>
-      </c>
-      <c r="F35" s="16" t="n">
-        <f aca="false">F20-F32</f>
-        <v>4274806.64122</v>
+      <c r="A35" s="4" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B36" s="15" t="n">
-        <f aca="false">B35</f>
-        <v>180969.64</v>
-      </c>
-      <c r="C36" s="15" t="n">
-        <f aca="false">B36+C35</f>
-        <v>661373.1</v>
-      </c>
-      <c r="D36" s="15" t="n">
-        <f aca="false">C36+D35</f>
-        <v>1869929.878</v>
-      </c>
-      <c r="E36" s="15" t="n">
-        <f aca="false">D36+E35</f>
-        <v>4325026.7294</v>
-      </c>
-      <c r="F36" s="15" t="n">
-        <f aca="false">E36+F35</f>
-        <v>8599833.37062</v>
+        <v>139</v>
+      </c>
+      <c r="B36" s="16" t="n">
+        <f aca="false">B20-B33</f>
+        <v>179769.64</v>
+      </c>
+      <c r="C36" s="16" t="n">
+        <f aca="false">C20-C33</f>
+        <v>479203.46</v>
+      </c>
+      <c r="D36" s="16" t="n">
+        <f aca="false">D20-D33</f>
+        <v>1207356.778</v>
+      </c>
+      <c r="E36" s="16" t="n">
+        <f aca="false">E20-E33</f>
+        <v>2453896.8514</v>
+      </c>
+      <c r="F36" s="16" t="n">
+        <f aca="false">F20-F33</f>
+        <v>4273606.64122</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B37" s="18" t="n">
-        <f aca="false">IF(B20=0,0,B35/B20)</f>
-        <v>0.858326882944413</v>
-      </c>
-      <c r="C37" s="18" t="n">
-        <f aca="false">IF(C20=0,0,C35/C20)</f>
-        <v>0.89751421738968</v>
-      </c>
-      <c r="D37" s="18" t="n">
-        <f aca="false">IF(D20=0,0,D35/D20)</f>
-        <v>0.922197770652521</v>
-      </c>
-      <c r="E37" s="18" t="n">
-        <f aca="false">IF(E20=0,0,E35/E20)</f>
-        <v>0.92648191876761</v>
-      </c>
-      <c r="F37" s="18" t="n">
-        <f aca="false">IF(F20=0,0,F35/F20)</f>
-        <v>0.933450755297575</v>
+        <v>140</v>
+      </c>
+      <c r="B37" s="15" t="n">
+        <f aca="false">B36</f>
+        <v>179769.64</v>
+      </c>
+      <c r="C37" s="15" t="n">
+        <f aca="false">B37+C36</f>
+        <v>658973.1</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <f aca="false">C37+D36</f>
+        <v>1866329.878</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <f aca="false">D37+E36</f>
+        <v>4320226.7294</v>
+      </c>
+      <c r="F37" s="15" t="n">
+        <f aca="false">E37+F36</f>
+        <v>8593833.37062</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B38" s="15" t="n">
+        <v>141</v>
+      </c>
+      <c r="B38" s="18" t="n">
+        <f aca="false">IF(B20=0,0,B36/B20)</f>
+        <v>0.85263536330867</v>
+      </c>
+      <c r="C38" s="18" t="n">
+        <f aca="false">IF(C20=0,0,C36/C20)</f>
+        <v>0.89527231625752</v>
+      </c>
+      <c r="D38" s="18" t="n">
+        <f aca="false">IF(D20=0,0,D36/D20)</f>
+        <v>0.921282102191652</v>
+      </c>
+      <c r="E38" s="18" t="n">
+        <f aca="false">IF(E20=0,0,E36/E20)</f>
+        <v>0.926029073780298</v>
+      </c>
+      <c r="F38" s="18" t="n">
+        <f aca="false">IF(F20=0,0,F36/F20)</f>
+        <v>0.93318872218114</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B39" s="15" t="n">
         <f aca="false">B20</f>
         <v>210840</v>
       </c>
-      <c r="C38" s="15" t="n">
+      <c r="C39" s="15" t="n">
         <f aca="false">C20</f>
         <v>535260</v>
       </c>
-      <c r="D38" s="15" t="n">
+      <c r="D39" s="15" t="n">
         <f aca="false">D20</f>
         <v>1310518</v>
       </c>
-      <c r="E38" s="15" t="n">
+      <c r="E39" s="15" t="n">
         <f aca="false">E20</f>
         <v>2649913.4</v>
       </c>
-      <c r="F38" s="15" t="n">
+      <c r="F39" s="15" t="n">
         <f aca="false">F20</f>
         <v>4579573.82</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
-        <v>137</v>
-      </c>
-    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B41" s="15" t="n">
+      <c r="A41" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B42" s="15" t="n">
         <f aca="false">F20</f>
         <v>4579573.82</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B42" s="6" t="n">
-        <v>20</v>
-      </c>
-    </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B43" s="16" t="n">
+        <v>145</v>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B44" s="16" t="n">
         <f aca="false">B41*B42</f>
-        <v>91591476.4</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="B45" s="16" t="n">
-        <f aca="false">B43*0.05</f>
-        <v>4579573.82</v>
-      </c>
-    </row>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="B46" s="19" t="n">
+        <v>147</v>
+      </c>
+      <c r="B46" s="16" t="n">
+        <f aca="false">B43*(50000/5050000)</f>
+        <v>0.198019801980198</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B47" s="19" t="n">
         <f aca="false">B45/50000</f>
-        <v>91.5914764</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="B49" s="1" t="n">
-        <v>80</v>
+      <c r="A49" s="4" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B50" s="1" t="n">
-        <v>58</v>
+        <v>100</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B51" s="1" t="n">
-        <v>20</v>
+        <v>72</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>148</v>
+        <v>152</v>
+      </c>
+      <c r="B52" s="1" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>